<commit_message>
Format cetak RPS OBE (Template FF UMI A–P) + logo kop, TTD elektronik, konfigurasi aturan superadmin
- Cetak/DOCX default format OBE formulir mutu (bagian A–P); format KPT 2024 via ?format=kpt
- Kelengkapan dokumen per RPS (tahun akademik, berlaku mulai, otorisasi, media/LMS/proporsi, peran CPL, lampiran) + PUT /rps-versions/{id}/kelengkapan
- Kolom pekanan Media/Sumber & Bukti/Produk (generator, editor, impor Excel, prompt)
- Referensi +standar/jurnal; konversi nilai huruf (konfigurasi skala_nilai)
- Logo institusi (warisan prodi→fakultas→universitas) di menu Logo & Kop Dokumen
- Spesimen TTD elektronik di Profil Saya, dibubuhkan otomatis setelah tahap persetujuan + kode verifikasi
- Superadmin memilih unit tujuan konfigurasi aturan; daftar aturan default ke institusi pengguna
- Prompt mingguan & penilaian diselaraskan dengan template OBE
</commit_message>
<xml_diff>
--- a/curriculum-web/public/template-impor-rps.xlsx
+++ b/curriculum-web/public/template-impor-rps.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="74">
   <si>
     <t>Template Impor RPS Lama</t>
   </si>
@@ -41,7 +41,7 @@
     <t>Sheet Sub-CPMK   : Kode | Kode CPMK Induk | Deskripsi | Taksonomi (pisah ;) | Indikator (pisah ;)</t>
   </si>
   <si>
-    <t>Sheet Mingguan   : Minggu | Kode Sub-CPMK | Indikator | Kriteria | Metode | Bentuk Luring | Bentuk Daring | Pengalaman | Materi/Pustaka | Bobot(%)</t>
+    <t>Sheet Mingguan   : Minggu | Kode Sub-CPMK | Indikator | Kriteria | Metode | Bentuk Luring | Bentuk Daring | Pengalaman | Materi/Pustaka | Bobot(%) | Media/Sumber | Bukti/Produk</t>
   </si>
   <si>
     <t>Sheet Penilaian  : Nama | Jenis | Bobot(%) | Kode Sub-CPMK | Minggu | Instrumen</t>
@@ -149,6 +149,12 @@
     <t>Bobot (%)</t>
   </si>
   <si>
+    <t>Media / Sumber</t>
+  </si>
+  <si>
+    <t>Bukti / Produk</t>
+  </si>
+  <si>
     <t>Ketepatan menjelaskan</t>
   </si>
   <si>
@@ -170,6 +176,12 @@
     <t>Farmakologi Dasar — Bab 1 [Pustaka: 1]</t>
   </si>
   <si>
+    <t>Slide, video</t>
+  </si>
+  <si>
+    <t>Ringkasan konsep</t>
+  </si>
+  <si>
     <t>Ketepatan analisis</t>
   </si>
   <si>
@@ -189,6 +201,12 @@
   </si>
   <si>
     <t>Bab 2 [Pustaka: 1,2]</t>
+  </si>
+  <si>
+    <t>Kasus tertulis [Pustaka: 2]</t>
+  </si>
+  <si>
+    <t>Laporan analisis kasus</t>
   </si>
   <si>
     <t>Nama Komponen</t>
@@ -810,7 +828,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
@@ -822,9 +840,10 @@
     <col min="8" max="8" width="22.7109375" customWidth="1"/>
     <col min="9" max="9" width="32.7109375" customWidth="1"/>
     <col min="10" max="10" width="9.7109375" customWidth="1"/>
+    <col min="11" max="12" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" s="3" t="s">
         <v>33</v>
       </c>
@@ -855,8 +874,14 @@
       <c r="J1" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -864,31 +889,37 @@
         <v>26</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J2" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -896,28 +927,34 @@
         <v>30</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J3" s="4">
         <v>5</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -940,10 +977,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>42</v>
@@ -955,15 +992,15 @@
         <v>33</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C2" s="4">
         <v>20</v>
@@ -975,15 +1012,15 @@
         <v>4</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C3" s="4">
         <v>30</v>
@@ -995,15 +1032,15 @@
         <v>8</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C4" s="4">
         <v>50</v>
@@ -1015,7 +1052,7 @@
         <v>16</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>